<commit_message>
Add WWTP approval routes and refactor existing routes
- Introduced new routes for WWTP approval functionalities in both api-wwtp-routes.php and wwtp-routes.php.
- Removed redundant POST routes for 'influent-harian' and 'ph-harian' in api-wwtp-routes.php.
- Organized and grouped approval-related routes under a new prefix 'wwtp-approval'.
- Ensured that all routes are properly linked to their respective controller methods for better maintainability.
</commit_message>
<xml_diff>
--- a/public/assets/templates/Template_wwtp.xlsx
+++ b/public/assets/templates/Template_wwtp.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ba7654d4822b2758/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E68C7588-B5A4-4F4C-B491-E082EF041CA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DF40314-C8FD-47C7-867F-2572B26FA2CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{3BDCFB87-4C6E-4120-841E-20396DB35135}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet 1'!$A$1:$P$50</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet 1'!$A$1:$P$51</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1025,7 +1025,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1093,6 +1093,36 @@
       <sz val="9"/>
       <name val="Times New Roman"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1102,7 +1132,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -1389,23 +1419,227 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1417,213 +1651,66 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1993,7 +2080,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA050746-D6F5-43D7-A081-B19BC7008E20}">
-  <dimension ref="B1:S50"/>
+  <dimension ref="B1:S51"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="29.54296875" customWidth="1"/>
@@ -2005,1175 +2092,1098 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15" thickBot="1"/>
     <row r="2" spans="2:18" ht="20">
-      <c r="B2" s="2"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="4" t="s">
+      <c r="B2" s="60"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="5" t="s">
+      <c r="E2" s="64"/>
+      <c r="F2" s="64"/>
+      <c r="G2" s="64"/>
+      <c r="H2" s="64"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="7"/>
+      <c r="N2" s="65"/>
+      <c r="O2" s="65"/>
+      <c r="P2" s="66"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
     </row>
     <row r="3" spans="2:18" ht="17.5">
-      <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="10" t="s">
+      <c r="B3" s="62"/>
+      <c r="C3" s="63"/>
+      <c r="D3" s="69" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10"/>
-      <c r="L3" s="10"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="7"/>
-      <c r="R3" s="7"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="69"/>
+      <c r="I3" s="69"/>
+      <c r="J3" s="69"/>
+      <c r="K3" s="69"/>
+      <c r="L3" s="69"/>
+      <c r="M3" s="67"/>
+      <c r="N3" s="67"/>
+      <c r="O3" s="67"/>
+      <c r="P3" s="68"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
     </row>
     <row r="4" spans="2:18" ht="15.5">
-      <c r="B4" s="8"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="14"/>
+      <c r="B4" s="62"/>
+      <c r="C4" s="63"/>
+      <c r="D4" s="63"/>
+      <c r="E4" s="63"/>
+      <c r="F4" s="63"/>
+      <c r="G4" s="63"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="63"/>
+      <c r="L4" s="63"/>
+      <c r="M4" s="63"/>
+      <c r="N4" s="63"/>
+      <c r="O4" s="63"/>
+      <c r="P4" s="70"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
     </row>
     <row r="5" spans="2:18">
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="73" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17" t="s">
+      <c r="E5" s="36"/>
+      <c r="F5" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17" t="s">
+      <c r="G5" s="36"/>
+      <c r="H5" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="17"/>
-      <c r="J5" s="18" t="s">
+      <c r="I5" s="36"/>
+      <c r="J5" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="19" t="s">
+      <c r="K5" s="59" t="s">
         <v>9</v>
       </c>
-      <c r="L5" s="19" t="s">
+      <c r="L5" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="M5" s="18" t="s">
+      <c r="M5" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="N5" s="19" t="s">
+      <c r="N5" s="59" t="s">
         <v>12</v>
       </c>
-      <c r="O5" s="19" t="s">
+      <c r="O5" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="P5" s="20" t="s">
+      <c r="P5" s="57" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6" spans="2:18">
-      <c r="B6" s="21"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="22"/>
-      <c r="O6" s="22"/>
-      <c r="P6" s="23"/>
+      <c r="B6" s="72"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="36"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="36"/>
+      <c r="H6" s="36"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="36"/>
+      <c r="K6" s="53"/>
+      <c r="L6" s="53"/>
+      <c r="M6" s="36"/>
+      <c r="N6" s="53"/>
+      <c r="O6" s="53"/>
+      <c r="P6" s="54"/>
     </row>
     <row r="7" spans="2:18">
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="26"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="22"/>
-      <c r="L7" s="22"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="22"/>
-      <c r="O7" s="22"/>
-      <c r="P7" s="23"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="42"/>
+      <c r="E7" s="42"/>
+      <c r="F7" s="42"/>
+      <c r="G7" s="42"/>
+      <c r="H7" s="42"/>
+      <c r="I7" s="42"/>
+      <c r="J7" s="36"/>
+      <c r="K7" s="53"/>
+      <c r="L7" s="53"/>
+      <c r="M7" s="36"/>
+      <c r="N7" s="53"/>
+      <c r="O7" s="53"/>
+      <c r="P7" s="54"/>
     </row>
     <row r="8" spans="2:18">
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="29" t="s">
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="36"/>
+      <c r="J8" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="K8" s="29"/>
-      <c r="L8" s="29"/>
-      <c r="M8" s="30"/>
-      <c r="N8" s="30"/>
-      <c r="O8" s="30"/>
-      <c r="P8" s="31"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="10"/>
     </row>
     <row r="9" spans="2:18">
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="29" t="s">
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="29"/>
-      <c r="L9" s="29"/>
-      <c r="M9" s="30"/>
-      <c r="N9" s="30"/>
-      <c r="O9" s="30"/>
-      <c r="P9" s="31"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
+      <c r="P9" s="10"/>
     </row>
     <row r="10" spans="2:18">
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="29" t="s">
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="36"/>
+      <c r="H10" s="36"/>
+      <c r="I10" s="36"/>
+      <c r="J10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="K10" s="29"/>
-      <c r="L10" s="29"/>
-      <c r="M10" s="30"/>
-      <c r="N10" s="30"/>
-      <c r="O10" s="30"/>
-      <c r="P10" s="31"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
+      <c r="O10" s="9"/>
+      <c r="P10" s="10"/>
     </row>
     <row r="11" spans="2:18">
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="29" t="s">
+      <c r="D11" s="36"/>
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="36"/>
+      <c r="J11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="K11" s="29"/>
-      <c r="L11" s="29"/>
-      <c r="M11" s="30"/>
-      <c r="N11" s="30"/>
-      <c r="O11" s="30"/>
-      <c r="P11" s="31"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="9"/>
+      <c r="P11" s="10"/>
     </row>
     <row r="12" spans="2:18">
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="29" t="s">
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="36"/>
+      <c r="I12" s="36"/>
+      <c r="J12" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="K12" s="29"/>
-      <c r="L12" s="29"/>
-      <c r="M12" s="30"/>
-      <c r="N12" s="30"/>
-      <c r="O12" s="30"/>
-      <c r="P12" s="31"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
+      <c r="O12" s="9"/>
+      <c r="P12" s="10"/>
     </row>
     <row r="13" spans="2:18">
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="28" t="s">
+      <c r="C13" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="29" t="s">
+      <c r="D13" s="36"/>
+      <c r="E13" s="36"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="36"/>
+      <c r="J13" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="K13" s="29"/>
-      <c r="L13" s="29"/>
-      <c r="M13" s="29"/>
-      <c r="N13" s="29"/>
-      <c r="O13" s="29"/>
-      <c r="P13" s="31"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="10"/>
     </row>
     <row r="14" spans="2:18" ht="17" customHeight="1">
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="28" t="s">
+      <c r="C14" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="33" t="s">
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="36"/>
+      <c r="I14" s="36"/>
+      <c r="J14" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="K14" s="34"/>
-      <c r="L14" s="34"/>
-      <c r="M14" s="34"/>
-      <c r="N14" s="34"/>
-      <c r="O14" s="34"/>
-      <c r="P14" s="35"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="13"/>
+      <c r="M14" s="13"/>
+      <c r="N14" s="13"/>
+      <c r="O14" s="13"/>
+      <c r="P14" s="14"/>
     </row>
     <row r="15" spans="2:18">
-      <c r="B15" s="24" t="s">
+      <c r="B15" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="36"/>
-      <c r="D15" s="37"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="37"/>
-      <c r="I15" s="37"/>
-      <c r="J15" s="38" t="s">
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K15" s="29"/>
-      <c r="L15" s="29"/>
-      <c r="M15" s="30"/>
-      <c r="N15" s="30"/>
-      <c r="O15" s="30"/>
-      <c r="P15" s="31"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="9"/>
+      <c r="P15" s="10"/>
     </row>
     <row r="16" spans="2:18" ht="15" customHeight="1">
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="28"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="39"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="39"/>
-      <c r="J16" s="40" t="s">
+      <c r="C16" s="4"/>
+      <c r="D16" s="40"/>
+      <c r="E16" s="41"/>
+      <c r="F16" s="40"/>
+      <c r="G16" s="41"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="41"/>
+      <c r="J16" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="K16" s="29"/>
-      <c r="L16" s="29"/>
-      <c r="M16" s="30"/>
-      <c r="N16" s="30"/>
-      <c r="O16" s="30"/>
-      <c r="P16" s="31"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+      <c r="O16" s="9"/>
+      <c r="P16" s="10"/>
     </row>
     <row r="17" spans="2:18">
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="39"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="39"/>
-      <c r="J17" s="41" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="40"/>
+      <c r="E17" s="41"/>
+      <c r="F17" s="40"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="40"/>
+      <c r="I17" s="41"/>
+      <c r="J17" s="55" t="s">
         <v>36</v>
       </c>
-      <c r="K17" s="22"/>
-      <c r="L17" s="22"/>
-      <c r="M17" s="22"/>
-      <c r="N17" s="22"/>
-      <c r="O17" s="22"/>
-      <c r="P17" s="23"/>
+      <c r="K17" s="53"/>
+      <c r="L17" s="53"/>
+      <c r="M17" s="53"/>
+      <c r="N17" s="53"/>
+      <c r="O17" s="53"/>
+      <c r="P17" s="54"/>
     </row>
     <row r="18" spans="2:18">
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="28"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="39"/>
-      <c r="J18" s="42"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="22"/>
-      <c r="P18" s="23"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="40"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="41"/>
+      <c r="H18" s="40"/>
+      <c r="I18" s="41"/>
+      <c r="J18" s="56"/>
+      <c r="K18" s="53"/>
+      <c r="L18" s="53"/>
+      <c r="M18" s="53"/>
+      <c r="N18" s="53"/>
+      <c r="O18" s="53"/>
+      <c r="P18" s="54"/>
     </row>
     <row r="19" spans="2:18">
-      <c r="B19" s="32" t="s">
+      <c r="B19" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="25"/>
-      <c r="I19" s="39"/>
-      <c r="J19" s="43" t="s">
+      <c r="C19" s="4"/>
+      <c r="D19" s="40"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="40"/>
+      <c r="G19" s="41"/>
+      <c r="H19" s="40"/>
+      <c r="I19" s="41"/>
+      <c r="J19" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="K19" s="44"/>
-      <c r="L19" s="44"/>
-      <c r="M19" s="44"/>
-      <c r="N19" s="44"/>
-      <c r="O19" s="44"/>
-      <c r="P19" s="45"/>
+      <c r="K19" s="20"/>
+      <c r="L19" s="20"/>
+      <c r="M19" s="20"/>
+      <c r="N19" s="20"/>
+      <c r="O19" s="20"/>
+      <c r="P19" s="21"/>
     </row>
     <row r="20" spans="2:18">
-      <c r="B20" s="32" t="s">
+      <c r="B20" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="28"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="39"/>
-      <c r="J20" s="43" t="s">
+      <c r="C20" s="4"/>
+      <c r="D20" s="40"/>
+      <c r="E20" s="41"/>
+      <c r="F20" s="40"/>
+      <c r="G20" s="41"/>
+      <c r="H20" s="40"/>
+      <c r="I20" s="41"/>
+      <c r="J20" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="K20" s="46"/>
-      <c r="L20" s="46"/>
-      <c r="M20" s="36"/>
-      <c r="N20" s="36"/>
-      <c r="O20" s="36"/>
-      <c r="P20" s="47"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
+      <c r="P20" s="23"/>
     </row>
     <row r="21" spans="2:18">
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="39"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="39"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="39"/>
-      <c r="J21" s="43" t="s">
+      <c r="C21" s="4"/>
+      <c r="D21" s="40"/>
+      <c r="E21" s="41"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="41"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="41"/>
+      <c r="J21" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="K21" s="43"/>
-      <c r="L21" s="44"/>
-      <c r="M21" s="48"/>
-      <c r="N21" s="48"/>
-      <c r="O21" s="48"/>
-      <c r="P21" s="45"/>
+      <c r="K21" s="19"/>
+      <c r="L21" s="20"/>
+      <c r="M21" s="24"/>
+      <c r="N21" s="24"/>
+      <c r="O21" s="24"/>
+      <c r="P21" s="21"/>
     </row>
     <row r="22" spans="2:18">
-      <c r="B22" s="32" t="s">
+      <c r="B22" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="28"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="39"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="39"/>
-      <c r="J22" s="43" t="s">
+      <c r="C22" s="4"/>
+      <c r="D22" s="40"/>
+      <c r="E22" s="41"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="41"/>
+      <c r="H22" s="40"/>
+      <c r="I22" s="41"/>
+      <c r="J22" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="K22" s="43"/>
-      <c r="L22" s="44"/>
-      <c r="M22" s="48"/>
-      <c r="N22" s="48"/>
-      <c r="O22" s="48"/>
-      <c r="P22" s="45"/>
+      <c r="K22" s="19"/>
+      <c r="L22" s="20"/>
+      <c r="M22" s="24"/>
+      <c r="N22" s="24"/>
+      <c r="O22" s="24"/>
+      <c r="P22" s="21"/>
     </row>
     <row r="23" spans="2:18">
-      <c r="B23" s="32" t="s">
+      <c r="B23" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="28"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="39"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="39"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="39"/>
-      <c r="J23" s="43" t="s">
+      <c r="C23" s="4"/>
+      <c r="D23" s="40"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="40"/>
+      <c r="G23" s="41"/>
+      <c r="H23" s="40"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="K23" s="46"/>
-      <c r="L23" s="46"/>
-      <c r="M23" s="36"/>
-      <c r="N23" s="36"/>
-      <c r="O23" s="36"/>
-      <c r="P23" s="47"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="15"/>
+      <c r="N23" s="15"/>
+      <c r="O23" s="15"/>
+      <c r="P23" s="23"/>
     </row>
     <row r="24" spans="2:18">
-      <c r="B24" s="32" t="s">
+      <c r="B24" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="28"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="39"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="39"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="39"/>
-      <c r="J24" s="49" t="s">
+      <c r="C24" s="4"/>
+      <c r="D24" s="40"/>
+      <c r="E24" s="41"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="41"/>
+      <c r="H24" s="40"/>
+      <c r="I24" s="41"/>
+      <c r="J24" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="K24" s="49"/>
-      <c r="L24" s="50"/>
-      <c r="M24" s="51"/>
-      <c r="N24" s="51"/>
-      <c r="O24" s="51"/>
-      <c r="P24" s="52"/>
+      <c r="K24" s="25"/>
+      <c r="L24" s="26"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="27"/>
+      <c r="P24" s="28"/>
     </row>
     <row r="25" spans="2:18">
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="28"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="39"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="39"/>
-      <c r="H25" s="25"/>
-      <c r="I25" s="26"/>
-      <c r="J25" s="53" t="s">
+      <c r="C25" s="4"/>
+      <c r="D25" s="40"/>
+      <c r="E25" s="41"/>
+      <c r="F25" s="40"/>
+      <c r="G25" s="41"/>
+      <c r="H25" s="40"/>
+      <c r="I25" s="42"/>
+      <c r="J25" s="50" t="s">
         <v>51</v>
       </c>
-      <c r="K25" s="53"/>
-      <c r="L25" s="53"/>
-      <c r="M25" s="53"/>
-      <c r="N25" s="53"/>
-      <c r="O25" s="53"/>
-      <c r="P25" s="54"/>
-      <c r="R25" s="55"/>
+      <c r="K25" s="50"/>
+      <c r="L25" s="50"/>
+      <c r="M25" s="50"/>
+      <c r="N25" s="50"/>
+      <c r="O25" s="50"/>
+      <c r="P25" s="51"/>
+      <c r="R25" s="29"/>
     </row>
     <row r="26" spans="2:18">
-      <c r="B26" s="56" t="s">
+      <c r="B26" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17" t="s">
+      <c r="C26" s="36"/>
+      <c r="D26" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="E26" s="17"/>
-      <c r="F26" s="17" t="s">
+      <c r="E26" s="36"/>
+      <c r="F26" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="G26" s="17"/>
-      <c r="H26" s="17" t="s">
+      <c r="G26" s="36"/>
+      <c r="H26" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="I26" s="25"/>
-      <c r="J26" s="53"/>
-      <c r="K26" s="53"/>
-      <c r="L26" s="53"/>
-      <c r="M26" s="53"/>
-      <c r="N26" s="53"/>
-      <c r="O26" s="53"/>
-      <c r="P26" s="54"/>
+      <c r="I26" s="40"/>
+      <c r="J26" s="50"/>
+      <c r="K26" s="50"/>
+      <c r="L26" s="50"/>
+      <c r="M26" s="50"/>
+      <c r="N26" s="50"/>
+      <c r="O26" s="50"/>
+      <c r="P26" s="51"/>
     </row>
     <row r="27" spans="2:18">
-      <c r="B27" s="56"/>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="17"/>
-      <c r="I27" s="25"/>
-      <c r="J27" s="53"/>
-      <c r="K27" s="53"/>
-      <c r="L27" s="53"/>
-      <c r="M27" s="53"/>
-      <c r="N27" s="53"/>
-      <c r="O27" s="53"/>
-      <c r="P27" s="54"/>
+      <c r="B27" s="52"/>
+      <c r="C27" s="36"/>
+      <c r="D27" s="36"/>
+      <c r="E27" s="36"/>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36"/>
+      <c r="I27" s="40"/>
+      <c r="J27" s="50"/>
+      <c r="K27" s="50"/>
+      <c r="L27" s="50"/>
+      <c r="M27" s="50"/>
+      <c r="N27" s="50"/>
+      <c r="O27" s="50"/>
+      <c r="P27" s="51"/>
     </row>
     <row r="28" spans="2:18">
-      <c r="B28" s="32" t="s">
+      <c r="B28" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="57"/>
-      <c r="E28" s="58"/>
-      <c r="F28" s="57"/>
-      <c r="G28" s="58"/>
-      <c r="H28" s="57"/>
-      <c r="I28" s="59"/>
-      <c r="J28" s="53"/>
-      <c r="K28" s="53"/>
-      <c r="L28" s="53"/>
-      <c r="M28" s="53"/>
-      <c r="N28" s="53"/>
-      <c r="O28" s="53"/>
-      <c r="P28" s="54"/>
+      <c r="D28" s="47"/>
+      <c r="E28" s="49"/>
+      <c r="F28" s="47"/>
+      <c r="G28" s="49"/>
+      <c r="H28" s="47"/>
+      <c r="I28" s="48"/>
+      <c r="J28" s="50"/>
+      <c r="K28" s="50"/>
+      <c r="L28" s="50"/>
+      <c r="M28" s="50"/>
+      <c r="N28" s="50"/>
+      <c r="O28" s="50"/>
+      <c r="P28" s="51"/>
     </row>
     <row r="29" spans="2:18">
-      <c r="B29" s="32" t="s">
+      <c r="B29" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D29" s="57"/>
-      <c r="E29" s="58"/>
-      <c r="F29" s="57"/>
-      <c r="G29" s="58"/>
-      <c r="H29" s="57"/>
-      <c r="I29" s="59"/>
-      <c r="J29" s="53"/>
-      <c r="K29" s="53"/>
-      <c r="L29" s="53"/>
-      <c r="M29" s="53"/>
-      <c r="N29" s="53"/>
-      <c r="O29" s="53"/>
-      <c r="P29" s="54"/>
+      <c r="D29" s="47"/>
+      <c r="E29" s="49"/>
+      <c r="F29" s="47"/>
+      <c r="G29" s="49"/>
+      <c r="H29" s="47"/>
+      <c r="I29" s="48"/>
+      <c r="J29" s="50"/>
+      <c r="K29" s="50"/>
+      <c r="L29" s="50"/>
+      <c r="M29" s="50"/>
+      <c r="N29" s="50"/>
+      <c r="O29" s="50"/>
+      <c r="P29" s="51"/>
     </row>
     <row r="30" spans="2:18">
-      <c r="B30" s="32" t="s">
+      <c r="B30" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="C30" s="28" t="s">
+      <c r="C30" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D30" s="57"/>
-      <c r="E30" s="58"/>
-      <c r="F30" s="57"/>
-      <c r="G30" s="58"/>
-      <c r="H30" s="57"/>
-      <c r="I30" s="59"/>
-      <c r="J30" s="53"/>
-      <c r="K30" s="53"/>
-      <c r="L30" s="53"/>
-      <c r="M30" s="53"/>
-      <c r="N30" s="53"/>
-      <c r="O30" s="53"/>
-      <c r="P30" s="54"/>
+      <c r="D30" s="47"/>
+      <c r="E30" s="49"/>
+      <c r="F30" s="47"/>
+      <c r="G30" s="49"/>
+      <c r="H30" s="47"/>
+      <c r="I30" s="48"/>
+      <c r="J30" s="50"/>
+      <c r="K30" s="50"/>
+      <c r="L30" s="50"/>
+      <c r="M30" s="50"/>
+      <c r="N30" s="50"/>
+      <c r="O30" s="50"/>
+      <c r="P30" s="51"/>
     </row>
     <row r="31" spans="2:18">
-      <c r="B31" s="60" t="s">
+      <c r="B31" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="C31" s="28" t="s">
+      <c r="C31" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D31" s="57"/>
-      <c r="E31" s="58"/>
-      <c r="F31" s="57"/>
-      <c r="G31" s="58"/>
-      <c r="H31" s="57"/>
-      <c r="I31" s="59"/>
-      <c r="J31" s="53"/>
-      <c r="K31" s="53"/>
-      <c r="L31" s="53"/>
-      <c r="M31" s="53"/>
-      <c r="N31" s="53"/>
-      <c r="O31" s="53"/>
-      <c r="P31" s="54"/>
+      <c r="D31" s="47"/>
+      <c r="E31" s="49"/>
+      <c r="F31" s="47"/>
+      <c r="G31" s="49"/>
+      <c r="H31" s="47"/>
+      <c r="I31" s="48"/>
+      <c r="J31" s="50"/>
+      <c r="K31" s="50"/>
+      <c r="L31" s="50"/>
+      <c r="M31" s="50"/>
+      <c r="N31" s="50"/>
+      <c r="O31" s="50"/>
+      <c r="P31" s="51"/>
     </row>
     <row r="32" spans="2:18">
-      <c r="B32" s="32" t="s">
+      <c r="B32" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C32" s="28" t="s">
+      <c r="C32" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D32" s="57"/>
-      <c r="E32" s="58"/>
-      <c r="F32" s="57"/>
-      <c r="G32" s="58"/>
-      <c r="H32" s="57"/>
-      <c r="I32" s="59"/>
-      <c r="J32" s="53"/>
-      <c r="K32" s="53"/>
-      <c r="L32" s="53"/>
-      <c r="M32" s="53"/>
-      <c r="N32" s="53"/>
-      <c r="O32" s="53"/>
-      <c r="P32" s="54"/>
+      <c r="D32" s="47"/>
+      <c r="E32" s="49"/>
+      <c r="F32" s="47"/>
+      <c r="G32" s="49"/>
+      <c r="H32" s="47"/>
+      <c r="I32" s="48"/>
+      <c r="J32" s="50"/>
+      <c r="K32" s="50"/>
+      <c r="L32" s="50"/>
+      <c r="M32" s="50"/>
+      <c r="N32" s="50"/>
+      <c r="O32" s="50"/>
+      <c r="P32" s="51"/>
     </row>
     <row r="33" spans="2:19">
-      <c r="B33" s="32" t="s">
+      <c r="B33" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D33" s="57"/>
-      <c r="E33" s="58"/>
-      <c r="F33" s="57"/>
-      <c r="G33" s="58"/>
-      <c r="H33" s="57"/>
-      <c r="I33" s="59"/>
-      <c r="J33" s="53"/>
-      <c r="K33" s="53"/>
-      <c r="L33" s="53"/>
-      <c r="M33" s="53"/>
-      <c r="N33" s="53"/>
-      <c r="O33" s="53"/>
-      <c r="P33" s="54"/>
+      <c r="D33" s="47"/>
+      <c r="E33" s="49"/>
+      <c r="F33" s="47"/>
+      <c r="G33" s="49"/>
+      <c r="H33" s="47"/>
+      <c r="I33" s="48"/>
+      <c r="J33" s="50"/>
+      <c r="K33" s="50"/>
+      <c r="L33" s="50"/>
+      <c r="M33" s="50"/>
+      <c r="N33" s="50"/>
+      <c r="O33" s="50"/>
+      <c r="P33" s="51"/>
     </row>
     <row r="34" spans="2:19">
-      <c r="B34" s="32" t="s">
+      <c r="B34" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C34" s="28" t="s">
+      <c r="C34" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D34" s="57"/>
-      <c r="E34" s="58"/>
-      <c r="F34" s="57"/>
-      <c r="G34" s="58"/>
-      <c r="H34" s="57"/>
-      <c r="I34" s="59"/>
-      <c r="J34" s="53"/>
-      <c r="K34" s="53"/>
-      <c r="L34" s="53"/>
-      <c r="M34" s="53"/>
-      <c r="N34" s="53"/>
-      <c r="O34" s="53"/>
-      <c r="P34" s="54"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="49"/>
+      <c r="F34" s="47"/>
+      <c r="G34" s="49"/>
+      <c r="H34" s="47"/>
+      <c r="I34" s="48"/>
+      <c r="J34" s="50"/>
+      <c r="K34" s="50"/>
+      <c r="L34" s="50"/>
+      <c r="M34" s="50"/>
+      <c r="N34" s="50"/>
+      <c r="O34" s="50"/>
+      <c r="P34" s="51"/>
     </row>
     <row r="35" spans="2:19">
-      <c r="B35" s="32" t="s">
+      <c r="B35" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="28" t="s">
+      <c r="C35" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D35" s="57"/>
-      <c r="E35" s="58"/>
-      <c r="F35" s="57"/>
-      <c r="G35" s="58"/>
-      <c r="H35" s="57"/>
-      <c r="I35" s="59"/>
-      <c r="J35" s="53"/>
-      <c r="K35" s="53"/>
-      <c r="L35" s="53"/>
-      <c r="M35" s="53"/>
-      <c r="N35" s="53"/>
-      <c r="O35" s="53"/>
-      <c r="P35" s="54"/>
+      <c r="D35" s="47"/>
+      <c r="E35" s="49"/>
+      <c r="F35" s="47"/>
+      <c r="G35" s="49"/>
+      <c r="H35" s="47"/>
+      <c r="I35" s="48"/>
+      <c r="J35" s="50"/>
+      <c r="K35" s="50"/>
+      <c r="L35" s="50"/>
+      <c r="M35" s="50"/>
+      <c r="N35" s="50"/>
+      <c r="O35" s="50"/>
+      <c r="P35" s="51"/>
     </row>
     <row r="36" spans="2:19">
-      <c r="B36" s="24" t="s">
+      <c r="B36" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C36" s="25"/>
-      <c r="D36" s="26"/>
-      <c r="E36" s="26"/>
-      <c r="F36" s="26"/>
-      <c r="G36" s="26"/>
-      <c r="H36" s="26"/>
-      <c r="I36" s="26"/>
-      <c r="J36" s="53"/>
-      <c r="K36" s="53"/>
-      <c r="L36" s="53"/>
-      <c r="M36" s="53"/>
-      <c r="N36" s="53"/>
-      <c r="O36" s="53"/>
-      <c r="P36" s="54"/>
+      <c r="C36" s="40"/>
+      <c r="D36" s="42"/>
+      <c r="E36" s="42"/>
+      <c r="F36" s="42"/>
+      <c r="G36" s="42"/>
+      <c r="H36" s="42"/>
+      <c r="I36" s="42"/>
+      <c r="J36" s="50"/>
+      <c r="K36" s="50"/>
+      <c r="L36" s="50"/>
+      <c r="M36" s="50"/>
+      <c r="N36" s="50"/>
+      <c r="O36" s="50"/>
+      <c r="P36" s="51"/>
     </row>
     <row r="37" spans="2:19">
-      <c r="B37" s="32" t="s">
+      <c r="B37" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C37" s="28" t="s">
+      <c r="C37" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D37" s="57"/>
-      <c r="E37" s="59"/>
-      <c r="F37" s="57"/>
-      <c r="G37" s="59"/>
-      <c r="H37" s="57"/>
-      <c r="I37" s="59"/>
-      <c r="J37" s="53"/>
-      <c r="K37" s="53"/>
-      <c r="L37" s="53"/>
-      <c r="M37" s="53"/>
-      <c r="N37" s="53"/>
-      <c r="O37" s="53"/>
-      <c r="P37" s="54"/>
+      <c r="D37" s="47"/>
+      <c r="E37" s="48"/>
+      <c r="F37" s="47"/>
+      <c r="G37" s="48"/>
+      <c r="H37" s="47"/>
+      <c r="I37" s="48"/>
+      <c r="J37" s="50"/>
+      <c r="K37" s="50"/>
+      <c r="L37" s="50"/>
+      <c r="M37" s="50"/>
+      <c r="N37" s="50"/>
+      <c r="O37" s="50"/>
+      <c r="P37" s="51"/>
     </row>
     <row r="38" spans="2:19">
-      <c r="B38" s="32" t="s">
+      <c r="B38" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="C38" s="61" t="s">
+      <c r="C38" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D38" s="57"/>
-      <c r="E38" s="59"/>
-      <c r="F38" s="57"/>
-      <c r="G38" s="59"/>
-      <c r="H38" s="57"/>
-      <c r="I38" s="59"/>
-      <c r="J38" s="53"/>
-      <c r="K38" s="53"/>
-      <c r="L38" s="53"/>
-      <c r="M38" s="53"/>
-      <c r="N38" s="53"/>
-      <c r="O38" s="53"/>
-      <c r="P38" s="54"/>
+      <c r="D38" s="47"/>
+      <c r="E38" s="48"/>
+      <c r="F38" s="47"/>
+      <c r="G38" s="48"/>
+      <c r="H38" s="47"/>
+      <c r="I38" s="48"/>
+      <c r="J38" s="50"/>
+      <c r="K38" s="50"/>
+      <c r="L38" s="50"/>
+      <c r="M38" s="50"/>
+      <c r="N38" s="50"/>
+      <c r="O38" s="50"/>
+      <c r="P38" s="51"/>
     </row>
     <row r="39" spans="2:19">
-      <c r="B39" s="24" t="s">
+      <c r="B39" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C39" s="25"/>
-      <c r="D39" s="26"/>
-      <c r="E39" s="26"/>
-      <c r="F39" s="26"/>
-      <c r="G39" s="26"/>
-      <c r="H39" s="26"/>
-      <c r="I39" s="26"/>
-      <c r="J39" s="53"/>
-      <c r="K39" s="53"/>
-      <c r="L39" s="53"/>
-      <c r="M39" s="53"/>
-      <c r="N39" s="53"/>
-      <c r="O39" s="53"/>
-      <c r="P39" s="54"/>
+      <c r="C39" s="40"/>
+      <c r="D39" s="42"/>
+      <c r="E39" s="42"/>
+      <c r="F39" s="42"/>
+      <c r="G39" s="42"/>
+      <c r="H39" s="42"/>
+      <c r="I39" s="42"/>
+      <c r="J39" s="50"/>
+      <c r="K39" s="50"/>
+      <c r="L39" s="50"/>
+      <c r="M39" s="50"/>
+      <c r="N39" s="50"/>
+      <c r="O39" s="50"/>
+      <c r="P39" s="51"/>
     </row>
     <row r="40" spans="2:19">
-      <c r="B40" s="27" t="s">
+      <c r="B40" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="C40" s="28" t="s">
+      <c r="C40" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D40" s="25"/>
-      <c r="E40" s="39"/>
-      <c r="F40" s="25"/>
-      <c r="G40" s="39"/>
-      <c r="H40" s="25"/>
-      <c r="I40" s="26"/>
-      <c r="J40" s="53"/>
-      <c r="K40" s="53"/>
-      <c r="L40" s="53"/>
-      <c r="M40" s="53"/>
-      <c r="N40" s="53"/>
-      <c r="O40" s="53"/>
-      <c r="P40" s="54"/>
-      <c r="Q40" s="7"/>
-      <c r="R40" s="7"/>
+      <c r="D40" s="40"/>
+      <c r="E40" s="41"/>
+      <c r="F40" s="40"/>
+      <c r="G40" s="41"/>
+      <c r="H40" s="40"/>
+      <c r="I40" s="42"/>
+      <c r="J40" s="50"/>
+      <c r="K40" s="50"/>
+      <c r="L40" s="50"/>
+      <c r="M40" s="50"/>
+      <c r="N40" s="50"/>
+      <c r="O40" s="50"/>
+      <c r="P40" s="51"/>
+      <c r="Q40" s="2"/>
+      <c r="R40" s="2"/>
     </row>
     <row r="41" spans="2:19">
-      <c r="B41" s="27" t="s">
+      <c r="B41" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="C41" s="28" t="s">
+      <c r="C41" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D41" s="25"/>
-      <c r="E41" s="39"/>
-      <c r="F41" s="25"/>
-      <c r="G41" s="39"/>
-      <c r="H41" s="25"/>
-      <c r="I41" s="26"/>
-      <c r="J41" s="53"/>
-      <c r="K41" s="53"/>
-      <c r="L41" s="53"/>
-      <c r="M41" s="53"/>
-      <c r="N41" s="53"/>
-      <c r="O41" s="53"/>
-      <c r="P41" s="54"/>
-      <c r="Q41" s="7"/>
-      <c r="R41" s="7"/>
+      <c r="D41" s="40"/>
+      <c r="E41" s="41"/>
+      <c r="F41" s="40"/>
+      <c r="G41" s="41"/>
+      <c r="H41" s="40"/>
+      <c r="I41" s="42"/>
+      <c r="J41" s="50"/>
+      <c r="K41" s="50"/>
+      <c r="L41" s="50"/>
+      <c r="M41" s="50"/>
+      <c r="N41" s="50"/>
+      <c r="O41" s="50"/>
+      <c r="P41" s="51"/>
+      <c r="Q41" s="2"/>
+      <c r="R41" s="2"/>
     </row>
     <row r="42" spans="2:19">
-      <c r="B42" s="27" t="s">
+      <c r="B42" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C42" s="28" t="s">
+      <c r="C42" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D42" s="25"/>
-      <c r="E42" s="39"/>
-      <c r="F42" s="25"/>
-      <c r="G42" s="39"/>
-      <c r="H42" s="25"/>
-      <c r="I42" s="26"/>
-      <c r="J42" s="53"/>
-      <c r="K42" s="53"/>
-      <c r="L42" s="53"/>
-      <c r="M42" s="53"/>
-      <c r="N42" s="53"/>
-      <c r="O42" s="53"/>
-      <c r="P42" s="54"/>
-      <c r="Q42" s="7"/>
-      <c r="R42" s="7"/>
+      <c r="D42" s="40"/>
+      <c r="E42" s="41"/>
+      <c r="F42" s="40"/>
+      <c r="G42" s="41"/>
+      <c r="H42" s="40"/>
+      <c r="I42" s="42"/>
+      <c r="J42" s="50"/>
+      <c r="K42" s="50"/>
+      <c r="L42" s="50"/>
+      <c r="M42" s="50"/>
+      <c r="N42" s="50"/>
+      <c r="O42" s="50"/>
+      <c r="P42" s="51"/>
+      <c r="Q42" s="2"/>
+      <c r="R42" s="2"/>
     </row>
     <row r="43" spans="2:19">
-      <c r="B43" s="27" t="s">
+      <c r="B43" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="C43" s="28" t="s">
+      <c r="C43" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D43" s="25"/>
-      <c r="E43" s="39"/>
-      <c r="F43" s="25"/>
-      <c r="G43" s="39"/>
-      <c r="H43" s="25"/>
-      <c r="I43" s="26"/>
-      <c r="J43" s="53"/>
-      <c r="K43" s="53"/>
-      <c r="L43" s="53"/>
-      <c r="M43" s="53"/>
-      <c r="N43" s="53"/>
-      <c r="O43" s="53"/>
-      <c r="P43" s="54"/>
-      <c r="Q43" s="7"/>
-      <c r="R43" s="7"/>
+      <c r="D43" s="40"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="40"/>
+      <c r="G43" s="41"/>
+      <c r="H43" s="40"/>
+      <c r="I43" s="42"/>
+      <c r="J43" s="50"/>
+      <c r="K43" s="50"/>
+      <c r="L43" s="50"/>
+      <c r="M43" s="50"/>
+      <c r="N43" s="50"/>
+      <c r="O43" s="50"/>
+      <c r="P43" s="51"/>
+      <c r="Q43" s="2"/>
+      <c r="R43" s="2"/>
     </row>
     <row r="44" spans="2:19">
-      <c r="B44" s="62"/>
-      <c r="C44" s="63"/>
-      <c r="D44" s="63"/>
-      <c r="E44" s="63"/>
-      <c r="F44" s="63"/>
-      <c r="G44" s="63"/>
-      <c r="H44" s="63"/>
-      <c r="I44" s="63"/>
-      <c r="J44" s="63"/>
-      <c r="K44" s="63"/>
-      <c r="L44" s="63"/>
-      <c r="M44" s="63"/>
-      <c r="N44" s="63"/>
-      <c r="O44" s="63"/>
-      <c r="P44" s="64"/>
+      <c r="B44" s="43"/>
+      <c r="C44" s="44"/>
+      <c r="D44" s="44"/>
+      <c r="E44" s="44"/>
+      <c r="F44" s="44"/>
+      <c r="G44" s="44"/>
+      <c r="H44" s="44"/>
+      <c r="I44" s="44"/>
+      <c r="J44" s="44"/>
+      <c r="K44" s="44"/>
+      <c r="L44" s="44"/>
+      <c r="M44" s="44"/>
+      <c r="N44" s="44"/>
+      <c r="O44" s="44"/>
+      <c r="P44" s="45"/>
     </row>
     <row r="45" spans="2:19">
-      <c r="B45" s="65" t="s">
+      <c r="B45" s="37" t="s">
         <v>72</v>
       </c>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17" t="s">
+      <c r="C45" s="36"/>
+      <c r="D45" s="36"/>
+      <c r="E45" s="36" t="s">
         <v>73</v>
       </c>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
-      <c r="I45" s="17"/>
-      <c r="J45" s="17" t="s">
+      <c r="F45" s="36"/>
+      <c r="G45" s="36"/>
+      <c r="H45" s="36"/>
+      <c r="I45" s="36"/>
+      <c r="J45" s="36" t="s">
         <v>74</v>
       </c>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17"/>
-      <c r="N45" s="17"/>
-      <c r="O45" s="17"/>
-      <c r="P45" s="66"/>
-      <c r="Q45" s="67"/>
-      <c r="R45" s="67"/>
-      <c r="S45" s="67"/>
+      <c r="K45" s="36"/>
+      <c r="L45" s="36"/>
+      <c r="M45" s="36"/>
+      <c r="N45" s="36"/>
+      <c r="O45" s="36"/>
+      <c r="P45" s="46"/>
+      <c r="Q45" s="31"/>
+      <c r="R45" s="31"/>
+      <c r="S45" s="31"/>
     </row>
     <row r="46" spans="2:19">
-      <c r="B46" s="68"/>
-      <c r="C46" s="17"/>
-      <c r="D46" s="17"/>
-      <c r="E46" s="69"/>
-      <c r="F46" s="69"/>
-      <c r="G46" s="69"/>
-      <c r="H46" s="69"/>
-      <c r="I46" s="69"/>
-      <c r="J46" s="69"/>
-      <c r="K46" s="69"/>
-      <c r="L46" s="69"/>
-      <c r="M46" s="69"/>
-      <c r="N46" s="69"/>
-      <c r="O46" s="69"/>
-      <c r="P46" s="70"/>
-      <c r="Q46" s="71"/>
-      <c r="R46" s="71"/>
-      <c r="S46" s="71"/>
+      <c r="B46" s="35"/>
+      <c r="C46" s="36"/>
+      <c r="D46" s="36"/>
+      <c r="E46" s="38"/>
+      <c r="F46" s="38"/>
+      <c r="G46" s="38"/>
+      <c r="H46" s="38"/>
+      <c r="I46" s="38"/>
+      <c r="J46" s="38"/>
+      <c r="K46" s="38"/>
+      <c r="L46" s="38"/>
+      <c r="M46" s="38"/>
+      <c r="N46" s="38"/>
+      <c r="O46" s="38"/>
+      <c r="P46" s="39"/>
+      <c r="Q46" s="32"/>
+      <c r="R46" s="32"/>
+      <c r="S46" s="32"/>
     </row>
     <row r="47" spans="2:19">
-      <c r="B47" s="65"/>
-      <c r="C47" s="17"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="69"/>
-      <c r="F47" s="69"/>
-      <c r="G47" s="69"/>
-      <c r="H47" s="69"/>
-      <c r="I47" s="69"/>
-      <c r="J47" s="69"/>
-      <c r="K47" s="69"/>
-      <c r="L47" s="69"/>
-      <c r="M47" s="69"/>
-      <c r="N47" s="69"/>
-      <c r="O47" s="69"/>
-      <c r="P47" s="70"/>
-      <c r="Q47" s="71"/>
-      <c r="R47" s="71"/>
-      <c r="S47" s="71"/>
+      <c r="B47" s="37"/>
+      <c r="C47" s="36"/>
+      <c r="D47" s="36"/>
+      <c r="E47" s="38"/>
+      <c r="F47" s="38"/>
+      <c r="G47" s="38"/>
+      <c r="H47" s="38"/>
+      <c r="I47" s="38"/>
+      <c r="J47" s="38"/>
+      <c r="K47" s="38"/>
+      <c r="L47" s="38"/>
+      <c r="M47" s="38"/>
+      <c r="N47" s="38"/>
+      <c r="O47" s="38"/>
+      <c r="P47" s="39"/>
+      <c r="Q47" s="32"/>
+      <c r="R47" s="32"/>
+      <c r="S47" s="32"/>
     </row>
     <row r="48" spans="2:19">
-      <c r="B48" s="65"/>
-      <c r="C48" s="17"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="69"/>
-      <c r="F48" s="69"/>
-      <c r="G48" s="69"/>
-      <c r="H48" s="69"/>
-      <c r="I48" s="69"/>
-      <c r="J48" s="69"/>
-      <c r="K48" s="69"/>
-      <c r="L48" s="69"/>
-      <c r="M48" s="69"/>
-      <c r="N48" s="69"/>
-      <c r="O48" s="69"/>
-      <c r="P48" s="70"/>
-      <c r="Q48" s="71"/>
-      <c r="R48" s="71"/>
-      <c r="S48" s="71"/>
-    </row>
-    <row r="49" spans="2:19" ht="15" thickBot="1">
-      <c r="B49" s="72" t="s">
+      <c r="B48" s="37"/>
+      <c r="C48" s="36"/>
+      <c r="D48" s="36"/>
+      <c r="E48" s="38"/>
+      <c r="F48" s="38"/>
+      <c r="G48" s="38"/>
+      <c r="H48" s="38"/>
+      <c r="I48" s="38"/>
+      <c r="J48" s="38"/>
+      <c r="K48" s="38"/>
+      <c r="L48" s="38"/>
+      <c r="M48" s="38"/>
+      <c r="N48" s="38"/>
+      <c r="O48" s="38"/>
+      <c r="P48" s="39"/>
+      <c r="Q48" s="32"/>
+      <c r="R48" s="32"/>
+      <c r="S48" s="32"/>
+    </row>
+    <row r="49" spans="2:19" s="74" customFormat="1">
+      <c r="B49" s="75" t="s">
         <v>75</v>
       </c>
-      <c r="C49" s="73"/>
-      <c r="D49" s="73"/>
-      <c r="E49" s="73" t="s">
+      <c r="C49" s="76"/>
+      <c r="D49" s="77"/>
+      <c r="E49" s="78" t="s">
         <v>76</v>
       </c>
-      <c r="F49" s="73"/>
-      <c r="G49" s="73"/>
-      <c r="H49" s="73"/>
-      <c r="I49" s="73"/>
-      <c r="J49" s="73" t="s">
+      <c r="F49" s="79"/>
+      <c r="G49" s="79"/>
+      <c r="H49" s="79"/>
+      <c r="I49" s="80"/>
+      <c r="J49" s="78" t="s">
         <v>77</v>
       </c>
-      <c r="K49" s="73"/>
-      <c r="L49" s="73"/>
-      <c r="M49" s="73"/>
-      <c r="N49" s="73"/>
-      <c r="O49" s="73"/>
-      <c r="P49" s="74"/>
-      <c r="Q49" s="75"/>
-      <c r="R49" s="75"/>
-      <c r="S49" s="75"/>
-    </row>
-    <row r="50" spans="2:19">
-      <c r="B50" s="67"/>
-      <c r="C50" s="67"/>
-      <c r="D50" s="67"/>
-      <c r="E50" s="67"/>
-      <c r="F50" s="67"/>
-      <c r="G50" s="67"/>
-      <c r="H50" s="67"/>
-      <c r="I50" s="67"/>
-      <c r="J50" s="67"/>
-      <c r="M50" s="76" t="s">
+      <c r="K49" s="79"/>
+      <c r="L49" s="79"/>
+      <c r="M49" s="79"/>
+      <c r="N49" s="79"/>
+      <c r="O49" s="79"/>
+      <c r="P49" s="81"/>
+      <c r="Q49" s="82"/>
+      <c r="R49" s="82"/>
+      <c r="S49" s="82"/>
+    </row>
+    <row r="50" spans="2:19" s="83" customFormat="1" ht="15" thickBot="1">
+      <c r="B50" s="84"/>
+      <c r="C50" s="85"/>
+      <c r="D50" s="85"/>
+      <c r="E50" s="85"/>
+      <c r="F50" s="85"/>
+      <c r="G50" s="85"/>
+      <c r="H50" s="85"/>
+      <c r="I50" s="85"/>
+      <c r="J50" s="85"/>
+      <c r="K50" s="85"/>
+      <c r="L50" s="85"/>
+      <c r="M50" s="85"/>
+      <c r="N50" s="85"/>
+      <c r="O50" s="85"/>
+      <c r="P50" s="86"/>
+      <c r="Q50" s="87"/>
+      <c r="R50" s="87"/>
+      <c r="S50" s="87"/>
+    </row>
+    <row r="51" spans="2:19">
+      <c r="B51" s="31"/>
+      <c r="C51" s="31"/>
+      <c r="D51" s="31"/>
+      <c r="E51" s="31"/>
+      <c r="F51" s="31"/>
+      <c r="G51" s="31"/>
+      <c r="H51" s="31"/>
+      <c r="I51" s="31"/>
+      <c r="J51" s="31"/>
+      <c r="M51" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="N50" s="76"/>
-      <c r="O50" s="76"/>
-      <c r="P50" s="76"/>
-      <c r="Q50" s="75"/>
-      <c r="R50" s="75"/>
+      <c r="N51" s="34"/>
+      <c r="O51" s="34"/>
+      <c r="P51" s="34"/>
+      <c r="Q51" s="33"/>
+      <c r="R51" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="137">
-    <mergeCell ref="M50:P50"/>
-    <mergeCell ref="B46:D48"/>
-    <mergeCell ref="E46:I48"/>
-    <mergeCell ref="J46:P48"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="E49:I49"/>
-    <mergeCell ref="J49:P49"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="B44:P44"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="E45:I45"/>
-    <mergeCell ref="J45:P45"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="C39:I39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="H40:I40"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="H35:I35"/>
-    <mergeCell ref="C36:I36"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="H37:I37"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="J25:P43"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:E27"/>
-    <mergeCell ref="F26:G27"/>
-    <mergeCell ref="H26:I27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="M17:M18"/>
-    <mergeCell ref="N17:N18"/>
-    <mergeCell ref="O17:O18"/>
-    <mergeCell ref="P17:P18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="K17:K18"/>
-    <mergeCell ref="L17:L18"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="H13:I13"/>
+  <mergeCells count="140">
+    <mergeCell ref="B2:C3"/>
+    <mergeCell ref="D2:L2"/>
+    <mergeCell ref="M2:P3"/>
+    <mergeCell ref="D3:L3"/>
+    <mergeCell ref="B4:P4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:E6"/>
+    <mergeCell ref="F5:G6"/>
+    <mergeCell ref="H5:I6"/>
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="H10:I10"/>
@@ -3194,16 +3204,116 @@
     <mergeCell ref="M5:M7"/>
     <mergeCell ref="N5:N7"/>
     <mergeCell ref="O5:O7"/>
-    <mergeCell ref="B2:C3"/>
-    <mergeCell ref="D2:L2"/>
-    <mergeCell ref="M2:P3"/>
-    <mergeCell ref="D3:L3"/>
-    <mergeCell ref="B4:P4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:E6"/>
-    <mergeCell ref="F5:G6"/>
-    <mergeCell ref="H5:I6"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="P17:P18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="K17:K18"/>
+    <mergeCell ref="L17:L18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="M17:M18"/>
+    <mergeCell ref="N17:N18"/>
+    <mergeCell ref="O17:O18"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="J25:P43"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:E27"/>
+    <mergeCell ref="F26:G27"/>
+    <mergeCell ref="H26:I27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="C36:I36"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="C39:I39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="M51:P51"/>
+    <mergeCell ref="B46:D48"/>
+    <mergeCell ref="E46:I48"/>
+    <mergeCell ref="J46:P48"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="E50:I50"/>
+    <mergeCell ref="J50:P50"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="B44:P44"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="E45:I45"/>
+    <mergeCell ref="J45:P45"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="E49:I49"/>
+    <mergeCell ref="J49:P49"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>